<commit_message>
Clean up workspace; close gaps in Lovable spec
- LOVABLE_PLAN: review_queue returns ReviewItem (latest completion + artifacts);
  server-side filters for board (person) and activity (via, kind); explicit
  mock-mode auto logic; route map, auth guard, polling and error design;
  UI defaults (theme, toasts, rail breakpoints, times, empty states);
  markdown without raw HTML; mock graph derived via buildGraph(); token-in-URL
  marked demo-only
- MVP_PLAN: API list aligned with the Lovable contract
- Remove superseded docs/PLAN.md; README rewritten; tracker regenerated for MVP
- Ignore local .claude/settings.local.json

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE3pdTgB4HhU3G279fbueC
</commit_message>
<xml_diff>
--- a/docs/Orchestra_Tracker.xlsx
+++ b/docs/Orchestra_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Team" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tasks'!$A$4:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tasks'!$A$4:$I$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -646,12 +646,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Permission engine: roles, clearance floor, task scope, allowed_actions</t>
+          <t>MVP plan + Lovable plan written, reviewed, merged</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>PLAN §1</t>
+          <t>MVP_PLAN</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr"/>
@@ -684,7 +684,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -694,27 +694,27 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>REST API (tasks, scope, docs, messages, overview, audit, admin)</t>
+          <t>New schema, 3-layer visibility rule, login + agent keys</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Hassan</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>PLAN §3</t>
+          <t>MVP_PLAN</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>MCP server (11 tools, bearer token = human's rights, audited as agent)</t>
+          <t>REST endpoints exactly matching LOVABLE_PLAN §4 (filters, review_queue, graph)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -747,17 +747,17 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>PLAN §2</t>
+          <t>LOVABLE §4</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -780,27 +780,27 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Seed: Northwind AI Adoption (8 users, 8 tasks, 6 docs); 23 tests</t>
+          <t>MCP tools: start/report/attach/submit, live agent presence, mention extraction</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Hassan</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>PLAN §5</t>
+          <t>MVP_PLAN</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
@@ -818,17 +818,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Fix GitHub access to omarjku/Orchestra so code can be pushed</t>
+          <t>Seed: Northwind project matching LOVABLE §7 (deps, mentions, live tasks)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>Hassan</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -838,10 +838,14 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr"/>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>LOVABLE §7</t>
+        </is>
+      </c>
       <c r="I9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
@@ -857,17 +861,17 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Everyone: npm install &amp;&amp; npm run dev locally; run npm test</t>
+          <t>Webhooks on task events (open-source integration story)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Hassan</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -877,12 +881,12 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>README</t>
+          <t>MVP_PLAN</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
@@ -900,17 +904,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Run cloudflared tunnel; give Saad the URL as VITE_API_URL</t>
+          <t>npm run sim: simulated agents John/Priya/Mia via real MCP</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>Hassan</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -920,12 +924,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>PLAN §4</t>
+          <t>MVP_PLAN</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
@@ -938,7 +942,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -948,7 +952,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Lovable: app shell, DEMO 'Log in as' switcher, Reset demo, 2s polling</t>
+          <t>Paste LOVABLE_PLAN into Lovable; shell, routes, login, mock mode</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -963,12 +967,12 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>PLAN §4</t>
+          <t>LOVABLE §10</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr"/>
@@ -981,7 +985,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -991,7 +995,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>My Work view: task cards by status, task detail, comments with 'via agent' badge</t>
+          <t>Board + task drawer (timeline, markdown, artifacts)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1006,12 +1010,12 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>PLAN §4</t>
+          <t>LOVABLE §5</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
@@ -1024,7 +1028,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1034,7 +1038,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Scope panel (people + docs) and Messages drawer</t>
+          <t>PM graph (react-force-graph-2d) with buildGraph() mock</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1049,12 +1053,12 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>PLAN §4</t>
+          <t>LOVABLE §6</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
@@ -1067,22 +1071,22 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Connect Claude Code to /mcp as Omar; run T-57 prompt; note tool friction</t>
+          <t>Activity, Knowledge, Review, Live agents rail</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>Saad</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1092,12 +1096,12 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>PLAN §2</t>
+          <t>LOVABLE §5</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
@@ -1110,22 +1114,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Improve MCP tool descriptions/outputs based on agent trial</t>
+          <t>Switch UI to LIVE; fix contract mismatches</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Hassan</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1135,10 +1139,14 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>LOVABLE §4</t>
+        </is>
+      </c>
       <c r="I16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1149,22 +1157,22 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Lead: Review queue + Mark done; scope editor with inline refusal messages</t>
+          <t>Connect Claude Code as a junior agent; run a task end-to-end</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Saad</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1174,14 +1182,10 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>PLAN §4</t>
-        </is>
-      </c>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1192,22 +1196,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Manager: Project overview (KPIs, milestone bars, blocked, people load)</t>
+          <t>Sim agents + real agent together; refusal moment works</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Saad</t>
+          <t>Hassan</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1217,14 +1221,10 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>PLAN §4</t>
-        </is>
-      </c>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1235,22 +1235,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Wire every button to allowed_actions; handle 403/404 messages in UI</t>
+          <t>Acceptance checklist (LOVABLE §9) 3x after reset</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>All</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1260,12 +1260,12 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>PLAN §3</t>
+          <t>LOVABLE §9</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr"/>
@@ -1278,17 +1278,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Add any endpoint fields Saad needs (keep contract in PLAN.md updated)</t>
+          <t>README: pitch, run steps, open source + integrations</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
@@ -1317,22 +1317,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Demo steps 1–4 pass end-to-end in browser + Claude Code</t>
+          <t>Record 2-min video</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Omar</t>
+          <t>All</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1342,14 +1342,10 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>PLAN §5</t>
-        </is>
-      </c>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1360,22 +1356,22 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Submission</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Admin: users &amp; roles table, full audit log with denied actions highlighted</t>
+          <t>ZIP repo + submit form</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Saad</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1385,296 +1381,15 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>PLAN §4</t>
-        </is>
-      </c>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>T19</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>A2 metrics on overview: agent actions, denied actions, review cycle time</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Hassan</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>T20</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Before/after workflow map + who owns each decision (README + slide)</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Hassan</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>01:30</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>T21</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Full demo 1–5 passes 3× clean after Reset demo</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Omar</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>02:00</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>PLAN §5</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>T22</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Bug-fix pass only; no new features</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>T23</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>README: run steps, MCP connect, permission model, disclosure (synthetic data)</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Omar</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>05:00</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>T24</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Demo</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Record 2-min video (no tokens/secrets on screen beyond demo tokens)</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>T25</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Submission</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>ZIP repo (no node_modules/data/.env) + submit Google Form</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Omar</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:I29"/>
-  <conditionalFormatting sqref="A5:I59">
+  <autoFilter ref="A4:I22"/>
+  <conditionalFormatting sqref="A5:I52">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="Completed"</formula>
     </cfRule>
@@ -1686,10 +1401,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Omar,Hassan,Saad,All"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1793,33 +1508,33 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Backend core</t>
+          <t>Plans agreed + merged</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Sat 26 Sep 18:45</t>
+          <t>Sat 26 Sep 20:30</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Permission engine, REST, MCP, seed data, 23 tests green</t>
+          <t>MVP_PLAN + LOVABLE_PLAN on main</t>
         </is>
       </c>
       <c r="E5" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A5)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A5)</f>
         <v/>
       </c>
       <c r="F5" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A5,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A5,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G5" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A5,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A5,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H5" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A5,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A5,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I5" s="6">
@@ -1839,33 +1554,33 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>UI screens + agent connected</t>
+          <t>Backend v1 matches LOVABLE_PLAN</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Sat 26 Sep 21:30</t>
+          <t>Sat 26 Sep 22:00</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Lovable UI on live API via tunnel; Claude Code connected as Omar's agent</t>
+          <t>All endpoints + MCP tools + tests green</t>
         </is>
       </c>
       <c r="E6" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A6)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A6)</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A6,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A6,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G6" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A6,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A6,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H6" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A6,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A6,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I6" s="6">
@@ -1885,33 +1600,33 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>DEMO PATH end-to-end</t>
+          <t>UI on mock data</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Sun 27 Sep 00:00</t>
+          <t>Sat 26 Sep 22:00</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Agent works T-57 → UI updates live → lead reviews → manager overview</t>
+          <t>All Lovable screens work in MOCK mode</t>
         </is>
       </c>
       <c r="E7" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A7)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A7)</f>
         <v/>
       </c>
       <c r="F7" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A7,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A7,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G7" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A7,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A7,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H7" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A7,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A7,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I7" s="6">
@@ -1931,33 +1646,33 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Admin, scope editor, audit, metrics — FEATURE FREEZE</t>
+          <t>LIVE end-to-end</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sun 27 Sep 02:00</t>
+          <t>Sun 27 Sep 00:30</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>All 5 demo steps work; refusals visible</t>
+          <t>UI on real API; sim agents + Claude Code agent visible live</t>
         </is>
       </c>
       <c r="E8" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A8)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A8)</f>
         <v/>
       </c>
       <c r="F8" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A8,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A8,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G8" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A8,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A8,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H8" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A8,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A8,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I8" s="6">
@@ -1977,33 +1692,33 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Demo polish — FEATURE FREEZE</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Sun 27 Sep 05:00</t>
+          <t>Sun 27 Sep 02:00</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Bug fixes only, 3 clean rehearsals, README</t>
+          <t>Acceptance checklist passes 3x after reset</t>
         </is>
       </c>
       <c r="E9" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A9)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A9)</f>
         <v/>
       </c>
       <c r="F9" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A9,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A9,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G9" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A9,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A9,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H9" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A9,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A9,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I9" s="6">
@@ -2033,23 +1748,23 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2-min video, ZIP repo, Google Form submitted</t>
+          <t>Video, ZIP, form submitted</t>
         </is>
       </c>
       <c r="E10" s="4">
-        <f>COUNTIF(Tasks!$B$5:$B$59,A10)</f>
+        <f>COUNTIF(Tasks!$B$5:$B$52,A10)</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A10,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A10,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="G10" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A10,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A10,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="H10" s="4">
-        <f>COUNTIFS(Tasks!$B$5:$B$59,A10,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$B$5:$B$52,A10,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="I10" s="6">
@@ -2090,7 +1805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2160,27 +1875,27 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Backend (permissions, MCP) → owns front↔back integration, agent demo, submission</t>
+          <t>Backend core (schema, REST, MCP) → integration, agent demo, submission</t>
         </is>
       </c>
       <c r="C4" s="4">
-        <f>COUNTIF(Tasks!$E$5:$E$59,A4)</f>
+        <f>COUNTIF(Tasks!$E$5:$E$52,A4)</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A4,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A4,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A4,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A4,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="F4" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A4,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A4,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="G4" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A4,Tasks!$F$5:$F$59,"Not started")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A4,Tasks!$F$5:$F$52,"Not started")</f>
         <v/>
       </c>
       <c r="H4" s="6">
@@ -2196,27 +1911,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Backend (REST, seed, metrics, MCP polish), workflow map</t>
+          <t>Seed data, webhooks, simulated agents, README</t>
         </is>
       </c>
       <c r="C5" s="4">
-        <f>COUNTIF(Tasks!$E$5:$E$59,A5)</f>
+        <f>COUNTIF(Tasks!$E$5:$E$52,A5)</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A5,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A5,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A5,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A5,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="F5" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A5,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A5,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="G5" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A5,Tasks!$F$5:$F$59,"Not started")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A5,Tasks!$F$5:$F$52,"Not started")</f>
         <v/>
       </c>
       <c r="H5" s="6">
@@ -2232,27 +1947,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Frontend in Lovable (all role views)</t>
+          <t>Lovable frontend per LOVABLE_PLAN.md</t>
         </is>
       </c>
       <c r="C6" s="4">
-        <f>COUNTIF(Tasks!$E$5:$E$59,A6)</f>
+        <f>COUNTIF(Tasks!$E$5:$E$52,A6)</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A6,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A6,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A6,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A6,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A6,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A6,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="G6" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A6,Tasks!$F$5:$F$59,"Not started")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A6,Tasks!$F$5:$F$52,"Not started")</f>
         <v/>
       </c>
       <c r="H6" s="6">
@@ -2272,23 +1987,23 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>COUNTIF(Tasks!$E$5:$E$59,A7)</f>
+        <f>COUNTIF(Tasks!$E$5:$E$52,A7)</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A7,Tasks!$F$5:$F$59,"Completed")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A7,Tasks!$F$5:$F$52,"Completed")</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A7,Tasks!$F$5:$F$59,"In progress")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A7,Tasks!$F$5:$F$52,"In progress")</f>
         <v/>
       </c>
       <c r="F7" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A7,Tasks!$F$5:$F$59,"Blocked")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A7,Tasks!$F$5:$F$52,"Blocked")</f>
         <v/>
       </c>
       <c r="G7" s="4">
-        <f>COUNTIFS(Tasks!$E$5:$E$59,A7,Tasks!$F$5:$F$59,"Not started")</f>
+        <f>COUNTIFS(Tasks!$E$5:$E$52,A7,Tasks!$F$5:$F$52,"Not started")</f>
         <v/>
       </c>
       <c r="H7" s="6">
@@ -2337,21 +2052,14 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>• M0 tasks were built by Claude in this session and are marked Completed; reassign if you want different owners on record.</t>
+          <t>• Source of truth: docs/MVP_PLAN.md (everyone) and docs/LOVABLE_PLAN.md (frontend + API contract).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>• Lovable preview can't reach localhost → use a cloudflared tunnel; Lovable must not add Supabase/auth (API is the only backend).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>• Targets are proposals against the 08:00 deadline; feature freeze 02:00.</t>
+          <t>• Feature freeze 02:00; after that bug fixes only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish Northwind demo data; update tracker
- Every task has a description and scope (the task drawer had empty
  sections; Omar's and Hassan's tasks are what real agents read)
- Removed "Senior-only task." notes from descriptions
- One believable overdue task: T-2 Architecture review (due 25 Sep, in
  progress) instead of T-7, which waits on the unfinished product API
- Fuller KB docs (brief, API conventions, brand voice, ADRs)
- New descriptions cross-reference tasks: 12 mention links in the PM graph (was 4)
- Tracker: T05, T06, T07 completed; T14 no longer mentions a refusal

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Orchestra_Tracker.xlsx
+++ b/docs/Orchestra_Tracker.xlsx
@@ -833,7 +833,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -846,7 +846,11 @@
           <t>LOVABLE §7</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>northwind.json polished: every task has a description + scope, fuller KB docs, 12 mention links in the graph, one believable overdue task (T-2).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -876,7 +880,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -889,7 +893,11 @@
           <t>MVP_PLAN</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Built in the backend rewrite: server/src/webhooks.ts, POST /api/webhooks (PM). Covered by api.test.ts.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -919,7 +927,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -932,7 +940,11 @@
           <t>MVP_PLAN</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>PR #6 merged. npm run sim (-- --reset). Agent scripts: server/sim/stories/northwind.json. Works hosted (--url) and with random keys.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1206,7 +1218,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Sim agents + real agent together; refusal moment works</t>
+          <t>Sim agents + real Claude Code agent together on the shared server (no staged refusal: team decision)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1307,7 +1319,11 @@
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Simulated agents section added (PR #6). Pitch + integrations still to do.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Tracker: T14 in progress (M3); sim notes for T07/T16
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Orchestra_Tracker.xlsx
+++ b/docs/Orchestra_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>PR #6 merged. npm run sim (-- --reset). Agent scripts: server/sim/stories/northwind.json. Works hosted (--url) and with random keys.</t>
+          <t>PRs #6 + #9 merged. Demo: npm run sim -- --reset --loop (agents stay active, redo work after Reset demo). Scripts: server/sim/stories/northwind.json. Hosted: --url; project file must match server PROJECT_FILE.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1237,7 +1237,11 @@
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Sim ready for this (--loop, --url). Next: run sim against the hosted URL + Hassan Claude Code agent (ak_hassan) on T-7 at the same time. Needs Railway URL from Omar; UI check needs T12.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1321,7 +1325,7 @@
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Simulated agents section added (PR #6). Pitch + integrations still to do.</t>
+          <t>Sim section added (PRs #6, #9: --loop, hosted runs). Pitch + integrations still to do.</t>
         </is>
       </c>
     </row>

</xml_diff>